<commit_message>
Student Info template (UP TO DATE)
</commit_message>
<xml_diff>
--- a/StdInfo.xlsx
+++ b/StdInfo.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carso\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Charles\Desktop\Fall'25\CS499\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA4998CE-67B1-4687-BD0D-E9F019F795DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5716EE1-5EBC-4D45-9A6C-E4F4E65F7079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Class 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Student Name</t>
   </si>
@@ -489,281 +489,32 @@
     <t>email sign off</t>
   </si>
   <si>
+    <t>Tony Stark</t>
+  </si>
+  <si>
+    <t>Howard Stark</t>
+  </si>
+  <si>
+    <t>howard@gmail.com</t>
+  </si>
+  <si>
+    <t>Howard Two</t>
+  </si>
+  <si>
     <t>Valerie Frizzle</t>
   </si>
   <si>
-    <t>Leonardo DiCaprio</t>
+    <t>Positive Taps</t>
   </si>
   <si>
-    <t>Arnold Schwarzenegger</t>
-  </si>
-  <si>
-    <t>Jim Carrey</t>
-  </si>
-  <si>
-    <t>Tom Cruise</t>
-  </si>
-  <si>
-    <t>Robert Downey Jr.</t>
-  </si>
-  <si>
-    <t>Emma Watson</t>
-  </si>
-  <si>
-    <t>Daniel Radcliffe</t>
-  </si>
-  <si>
-    <t>Chris Evans</t>
-  </si>
-  <si>
-    <t>Brad Pitt</t>
-  </si>
-  <si>
-    <t>Morgan Freeman</t>
-  </si>
-  <si>
-    <t>Tom Hanks</t>
-  </si>
-  <si>
-    <t>Hugh Jackman</t>
-  </si>
-  <si>
-    <t>Matt Damon</t>
-  </si>
-  <si>
-    <t>Will Smith</t>
-  </si>
-  <si>
-    <t>Cameron Diaz</t>
-  </si>
-  <si>
-    <t>Kate Winslet</t>
-  </si>
-  <si>
-    <t>Natalie Portman</t>
-  </si>
-  <si>
-    <t>Angelina Jolie</t>
-  </si>
-  <si>
-    <t>Adam Sandler</t>
-  </si>
-  <si>
-    <t>Anne Hathaway</t>
-  </si>
-  <si>
-    <t>Taylor Swift</t>
-  </si>
-  <si>
-    <t>Keira Knightley</t>
-  </si>
-  <si>
-    <t>Will Ferrell</t>
-  </si>
-  <si>
-    <t>Jack Black</t>
-  </si>
-  <si>
-    <t>Selena Gomez</t>
-  </si>
-  <si>
-    <t>Jennifer Aniston</t>
-  </si>
-  <si>
-    <t>Rachel McAdams</t>
-  </si>
-  <si>
-    <t>Heath Ledger</t>
-  </si>
-  <si>
-    <t>Scarlett Johansson</t>
-  </si>
-  <si>
-    <t>Keanu Reeves</t>
-  </si>
-  <si>
-    <t>George DiCaprio</t>
-  </si>
-  <si>
-    <t>Aurelia Schwarzenegger</t>
-  </si>
-  <si>
-    <t>Percy Carrey</t>
-  </si>
-  <si>
-    <t>Thomas Cruise</t>
-  </si>
-  <si>
-    <t>Elsie Downey</t>
-  </si>
-  <si>
-    <t>Chris Watson</t>
-  </si>
-  <si>
-    <t>Alan Radcliffe</t>
-  </si>
-  <si>
-    <t>Lisa Evans</t>
-  </si>
-  <si>
-    <t>William Pitt</t>
-  </si>
-  <si>
-    <t>Amos Hanks</t>
-  </si>
-  <si>
-    <t>Christopher Jackman</t>
-  </si>
-  <si>
-    <t>Kent Damon</t>
-  </si>
-  <si>
-    <t>Willard Smith</t>
-  </si>
-  <si>
-    <t>Emilio Diaz</t>
-  </si>
-  <si>
-    <t>Roger Winslet</t>
-  </si>
-  <si>
-    <t>Avner Hershlag</t>
-  </si>
-  <si>
-    <t>Marcheline Bertrand</t>
-  </si>
-  <si>
-    <t>Judy Sandler</t>
-  </si>
-  <si>
-    <t>Gerald Hathaway</t>
-  </si>
-  <si>
-    <t>Scott Swift</t>
-  </si>
-  <si>
-    <t>Will Knightley</t>
-  </si>
-  <si>
-    <t>Roy Ferrel</t>
-  </si>
-  <si>
-    <t>Judith Cohen</t>
-  </si>
-  <si>
-    <t>Ricardo Gomez</t>
-  </si>
-  <si>
-    <t>John Aniston</t>
-  </si>
-  <si>
-    <t>Lance McAdams</t>
-  </si>
-  <si>
-    <t>Kim Ledger</t>
-  </si>
-  <si>
-    <t>Karsten Johansson</t>
-  </si>
-  <si>
-    <t>Samuel Reeves</t>
-  </si>
-  <si>
-    <t>leonardo.parent@gmail.com</t>
-  </si>
-  <si>
-    <t>arnoldsparent123@gmail.com</t>
-  </si>
-  <si>
-    <t>carreyparrent@gmail.com</t>
-  </si>
-  <si>
-    <t>tomsparent@gmail.com</t>
-  </si>
-  <si>
-    <t>roberts.parent23@gmail.com</t>
-  </si>
-  <si>
-    <t>emmasparent004@gmail.com</t>
-  </si>
-  <si>
-    <t>danielleradcliffeparent@gmail.com</t>
-  </si>
-  <si>
-    <t>evans.parent33@gmail.com</t>
-  </si>
-  <si>
-    <t>bradpittsparent@gmail.com</t>
-  </si>
-  <si>
-    <t>freeman.parent45@gmail.com</t>
-  </si>
-  <si>
-    <t>tom.hanksparent@gmail.com</t>
-  </si>
-  <si>
-    <t>hughjackmanparent@gmail.com</t>
-  </si>
-  <si>
-    <t>matt.parent@gmail.com</t>
-  </si>
-  <si>
-    <t>willsmithsparent77@gmail.com</t>
-  </si>
-  <si>
-    <t>diazparent22@gmail.com</t>
-  </si>
-  <si>
-    <t>winslet.parent99@gmail.com</t>
-  </si>
-  <si>
-    <t>natalieparent34@gmail.com</t>
-  </si>
-  <si>
-    <t>angelinajolieparent@gmail.com</t>
-  </si>
-  <si>
-    <t>sandler.parent@gmail.com</t>
-  </si>
-  <si>
-    <t>hathawayparent64@gmail.com</t>
-  </si>
-  <si>
-    <t>taylorswiftparent@gmail.com</t>
-  </si>
-  <si>
-    <t>kiera.parent@gmail.com</t>
-  </si>
-  <si>
-    <t>willferrellparent@gmail.com</t>
-  </si>
-  <si>
-    <t>jack.blackparent@gmail.com</t>
-  </si>
-  <si>
-    <t>selenagomezparent78@gmail.com</t>
-  </si>
-  <si>
-    <t>jennifer.anistonparent@gmail.com</t>
-  </si>
-  <si>
-    <t>rachelparen88@gmail.com</t>
-  </si>
-  <si>
-    <t>heath.ledgerparent@gmail.com</t>
-  </si>
-  <si>
-    <t>johanssonparent008@gmail.com</t>
-  </si>
-  <si>
-    <t>keanureevesparent456@gmail.com</t>
+    <t>Negative Taps</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -791,10 +542,6 @@
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Comfortaa"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
@@ -826,7 +573,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -939,12 +686,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEAD1DC"/>
         <bgColor rgb="FFEAD1DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -1276,9 +1017,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1351,20 +1092,13 @@
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="17" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1385,26 +1119,45 @@
     <xf numFmtId="0" fontId="2" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1621,16 +1374,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:P1001"/>
   <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" customWidth="1"/>
-    <col min="3" max="3" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="3" width="16.88671875" customWidth="1"/>
+    <col min="4" max="4" width="24.88671875" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="26.5546875" customWidth="1"/>
     <col min="8" max="8" width="16.6640625" customWidth="1"/>
@@ -1658,20 +1410,24 @@
       <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="J1" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="23" t="s">
+      <c r="K1" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="27" t="s">
+      <c r="L1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
       <c r="O1" s="8"/>
@@ -1679,723 +1435,556 @@
     </row>
     <row r="2" spans="1:16" ht="14.4" thickTop="1" thickBot="1">
       <c r="A2" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="12" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
-      <c r="D2" s="39" t="s">
-        <v>73</v>
+      <c r="D2" s="35" t="s">
+        <v>15</v>
       </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="24" t="s">
-        <v>13</v>
+      <c r="E2" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="F2" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="26">
+      <c r="K2" s="26">
         <v>305</v>
       </c>
-      <c r="J2" s="28"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
+      <c r="L2" s="28"/>
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
       <c r="O2" s="8"/>
       <c r="P2" s="9"/>
     </row>
-    <row r="3" spans="1:16" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A3" s="15" t="s">
-        <v>15</v>
-      </c>
+    <row r="3" spans="1:16" ht="15.75" customHeight="1" thickTop="1">
+      <c r="A3" s="15"/>
       <c r="B3" s="16"/>
-      <c r="C3" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>74</v>
-      </c>
+      <c r="C3" s="17"/>
+      <c r="D3" s="18"/>
       <c r="E3" s="19"/>
       <c r="F3" s="20"/>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
       <c r="I3" s="7"/>
       <c r="K3" s="8"/>
-      <c r="L3" s="40" t="s">
-        <v>9</v>
-      </c>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="41"/>
-      <c r="P3" s="42"/>
-    </row>
-    <row r="4" spans="1:16" ht="13.8" thickTop="1">
-      <c r="A4" s="15" t="s">
-        <v>16</v>
-      </c>
+    </row>
+    <row r="4" spans="1:16" ht="13.8" customHeight="1">
+      <c r="A4" s="15"/>
       <c r="B4" s="16"/>
-      <c r="C4" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="C4" s="17"/>
+      <c r="D4" s="18"/>
       <c r="E4" s="19"/>
       <c r="F4" s="20"/>
-      <c r="G4" s="7"/>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
       <c r="K4" s="8"/>
-      <c r="L4" s="43" t="s">
-        <v>11</v>
-      </c>
-      <c r="M4" s="44"/>
-      <c r="N4" s="44"/>
-      <c r="O4" s="44"/>
-      <c r="P4" s="45"/>
     </row>
     <row r="5" spans="1:16" ht="13.2">
-      <c r="A5" s="15" t="s">
-        <v>17</v>
-      </c>
+      <c r="A5" s="15"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>76</v>
-      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="18"/>
       <c r="E5" s="19"/>
       <c r="F5" s="20"/>
-      <c r="G5" s="7"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="46"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="47"/>
-      <c r="O5" s="47"/>
-      <c r="P5" s="48"/>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:16" ht="13.2">
-      <c r="A6" s="15" t="s">
-        <v>18</v>
-      </c>
+      <c r="A6" s="15"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>77</v>
-      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
       <c r="E6" s="19"/>
       <c r="F6" s="20"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="30"/>
-      <c r="L6" s="46"/>
-      <c r="M6" s="47"/>
-      <c r="N6" s="47"/>
-      <c r="O6" s="47"/>
-      <c r="P6" s="48"/>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:16" ht="13.2">
-      <c r="A7" s="15" t="s">
-        <v>19</v>
-      </c>
+      <c r="A7" s="15"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>78</v>
-      </c>
+      <c r="C7" s="17"/>
+      <c r="D7" s="18"/>
       <c r="E7" s="19"/>
       <c r="F7" s="20"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="29"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="46"/>
-      <c r="M7" s="47"/>
-      <c r="N7" s="47"/>
-      <c r="O7" s="47"/>
-      <c r="P7" s="48"/>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:16" ht="13.2">
-      <c r="A8" s="15" t="s">
-        <v>20</v>
-      </c>
+      <c r="A8" s="15"/>
       <c r="B8" s="16"/>
-      <c r="C8" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>79</v>
-      </c>
+      <c r="C8" s="17"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="19"/>
       <c r="F8" s="20"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="46"/>
-      <c r="M8" s="47"/>
-      <c r="N8" s="47"/>
-      <c r="O8" s="47"/>
-      <c r="P8" s="48"/>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:16" ht="13.2">
-      <c r="A9" s="15" t="s">
-        <v>21</v>
-      </c>
+      <c r="A9" s="15"/>
       <c r="B9" s="16"/>
-      <c r="C9" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>80</v>
-      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="19"/>
       <c r="F9" s="20"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="46"/>
-      <c r="M9" s="47"/>
-      <c r="N9" s="47"/>
-      <c r="O9" s="47"/>
-      <c r="P9" s="48"/>
-    </row>
-    <row r="10" spans="1:16" ht="15.6">
-      <c r="A10" s="15" t="s">
-        <v>22</v>
+      <c r="G9">
+        <v>0</v>
       </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="13.2">
+      <c r="A10" s="15"/>
       <c r="B10" s="16"/>
-      <c r="C10" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>81</v>
-      </c>
+      <c r="C10" s="17"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="19"/>
       <c r="F10" s="20"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="47"/>
-      <c r="N10" s="47"/>
-      <c r="O10" s="47"/>
-      <c r="P10" s="48"/>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:16" ht="13.2">
-      <c r="A11" s="15" t="s">
-        <v>23</v>
-      </c>
+      <c r="A11" s="15"/>
       <c r="B11" s="16"/>
-      <c r="C11" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>82</v>
-      </c>
+      <c r="C11" s="17"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="19"/>
       <c r="F11" s="20"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
-      <c r="L11" s="46"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="47"/>
-      <c r="P11" s="48"/>
     </row>
     <row r="12" spans="1:16" ht="13.2">
-      <c r="A12" s="15" t="s">
-        <v>24</v>
-      </c>
+      <c r="A12" s="15"/>
       <c r="B12" s="16"/>
-      <c r="C12" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>83</v>
-      </c>
+      <c r="C12" s="17"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="19"/>
       <c r="F12" s="20"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
-      <c r="L12" s="46"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="47"/>
-      <c r="P12" s="48"/>
     </row>
     <row r="13" spans="1:16" ht="13.2">
-      <c r="A13" s="15" t="s">
-        <v>25</v>
-      </c>
+      <c r="A13" s="15"/>
       <c r="B13" s="16"/>
-      <c r="C13" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>84</v>
-      </c>
+      <c r="C13" s="17"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
       <c r="I13" s="7"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
-      <c r="L13" s="46"/>
-      <c r="M13" s="47"/>
-      <c r="N13" s="47"/>
-      <c r="O13" s="47"/>
-      <c r="P13" s="48"/>
     </row>
     <row r="14" spans="1:16" ht="13.2">
-      <c r="A14" s="15" t="s">
-        <v>26</v>
-      </c>
+      <c r="A14" s="15"/>
       <c r="B14" s="16"/>
-      <c r="C14" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>85</v>
-      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="19"/>
       <c r="F14" s="20"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="47"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="47"/>
-      <c r="P14" s="48"/>
     </row>
     <row r="15" spans="1:16" ht="13.2">
-      <c r="A15" s="15" t="s">
-        <v>27</v>
-      </c>
+      <c r="A15" s="15"/>
       <c r="B15" s="16"/>
-      <c r="C15" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>86</v>
-      </c>
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="19"/>
       <c r="F15" s="20"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
       <c r="I15" s="7"/>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
-      <c r="L15" s="46"/>
-      <c r="M15" s="47"/>
-      <c r="N15" s="47"/>
-      <c r="O15" s="47"/>
-      <c r="P15" s="48"/>
     </row>
     <row r="16" spans="1:16" ht="13.2">
-      <c r="A16" s="15" t="s">
-        <v>28</v>
-      </c>
+      <c r="A16" s="15"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>87</v>
-      </c>
+      <c r="C16" s="17"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="19"/>
       <c r="F16" s="20"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
-      <c r="L16" s="46"/>
-      <c r="M16" s="47"/>
-      <c r="N16" s="47"/>
-      <c r="O16" s="47"/>
-      <c r="P16" s="48"/>
     </row>
     <row r="17" spans="1:16" ht="13.2">
-      <c r="A17" s="15" t="s">
-        <v>29</v>
-      </c>
+      <c r="A17" s="15"/>
       <c r="B17" s="16"/>
-      <c r="C17" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>88</v>
-      </c>
+      <c r="C17" s="17"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="19"/>
       <c r="F17" s="20"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
-      <c r="L17" s="46"/>
-      <c r="M17" s="47"/>
-      <c r="N17" s="47"/>
-      <c r="O17" s="47"/>
-      <c r="P17" s="48"/>
     </row>
     <row r="18" spans="1:16" ht="13.2">
-      <c r="A18" s="15" t="s">
-        <v>30</v>
-      </c>
+      <c r="A18" s="15"/>
       <c r="B18" s="16"/>
-      <c r="C18" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>89</v>
-      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" s="18"/>
       <c r="E18" s="19"/>
       <c r="F18" s="20"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
-      <c r="L18" s="46"/>
-      <c r="M18" s="47"/>
-      <c r="N18" s="47"/>
-      <c r="O18" s="47"/>
-      <c r="P18" s="48"/>
     </row>
     <row r="19" spans="1:16" ht="13.2">
-      <c r="A19" s="15" t="s">
-        <v>31</v>
-      </c>
+      <c r="A19" s="15"/>
       <c r="B19" s="16"/>
-      <c r="C19" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>90</v>
-      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="18"/>
       <c r="E19" s="19"/>
       <c r="F19" s="20"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
       <c r="I19" s="7"/>
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
-      <c r="L19" s="46"/>
-      <c r="M19" s="47"/>
-      <c r="N19" s="47"/>
-      <c r="O19" s="47"/>
-      <c r="P19" s="48"/>
     </row>
     <row r="20" spans="1:16" ht="13.2">
-      <c r="A20" s="15" t="s">
-        <v>32</v>
-      </c>
+      <c r="A20" s="15"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>91</v>
-      </c>
+      <c r="C20" s="17"/>
+      <c r="D20" s="18"/>
       <c r="E20" s="19"/>
       <c r="F20" s="20"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
       <c r="I20" s="7"/>
       <c r="J20" s="7"/>
       <c r="K20" s="7"/>
-      <c r="L20" s="46"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="47"/>
-      <c r="O20" s="47"/>
-      <c r="P20" s="48"/>
     </row>
     <row r="21" spans="1:16" ht="13.2">
-      <c r="A21" s="15" t="s">
-        <v>33</v>
-      </c>
+      <c r="A21" s="15"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>92</v>
-      </c>
+      <c r="C21" s="17"/>
+      <c r="D21" s="18"/>
       <c r="E21" s="19"/>
       <c r="F21" s="20"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
       <c r="I21" s="7"/>
       <c r="J21" s="7"/>
       <c r="K21" s="7"/>
-      <c r="L21" s="46"/>
-      <c r="M21" s="47"/>
-      <c r="N21" s="47"/>
-      <c r="O21" s="47"/>
-      <c r="P21" s="48"/>
     </row>
     <row r="22" spans="1:16" ht="13.2">
-      <c r="A22" s="15" t="s">
-        <v>34</v>
-      </c>
+      <c r="A22" s="15"/>
       <c r="B22" s="16"/>
-      <c r="C22" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>93</v>
-      </c>
+      <c r="C22" s="17"/>
+      <c r="D22" s="18"/>
       <c r="E22" s="19"/>
       <c r="F22" s="20"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
       <c r="I22" s="7"/>
       <c r="J22" s="7"/>
       <c r="K22" s="7"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="47"/>
-      <c r="P22" s="48"/>
-    </row>
-    <row r="23" spans="1:16" ht="13.2">
-      <c r="A23" s="15" t="s">
-        <v>35</v>
-      </c>
+    </row>
+    <row r="23" spans="1:16" ht="13.8" thickBot="1">
+      <c r="A23" s="15"/>
       <c r="B23" s="16"/>
-      <c r="C23" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="D23" s="18" t="s">
-        <v>94</v>
-      </c>
+      <c r="C23" s="17"/>
+      <c r="D23" s="18"/>
       <c r="E23" s="19"/>
       <c r="F23" s="20"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
-      <c r="L23" s="49"/>
-      <c r="M23" s="50"/>
-      <c r="N23" s="50"/>
-      <c r="O23" s="50"/>
-      <c r="P23" s="51"/>
-    </row>
-    <row r="24" spans="1:16" ht="13.2">
-      <c r="A24" s="15" t="s">
-        <v>36</v>
-      </c>
+    </row>
+    <row r="24" spans="1:16" ht="22.2" thickTop="1" thickBot="1">
+      <c r="A24" s="15"/>
       <c r="B24" s="16"/>
-      <c r="C24" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>95</v>
-      </c>
+      <c r="C24" s="17"/>
+      <c r="D24" s="18"/>
       <c r="E24" s="19"/>
       <c r="F24" s="20"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
+      <c r="K24" s="36" t="s">
+        <v>9</v>
+      </c>
+      <c r="L24" s="46"/>
+      <c r="M24" s="46"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="47"/>
       <c r="P24" s="9"/>
     </row>
-    <row r="25" spans="1:16" ht="13.2">
-      <c r="A25" s="15" t="s">
-        <v>37</v>
-      </c>
+    <row r="25" spans="1:16" ht="13.8" thickTop="1">
+      <c r="A25" s="15"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="D25" s="18" t="s">
-        <v>96</v>
-      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="18"/>
       <c r="E25" s="19"/>
       <c r="F25" s="20"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
+      <c r="K25" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="L25" s="38"/>
+      <c r="M25" s="38"/>
+      <c r="N25" s="38"/>
+      <c r="O25" s="39"/>
       <c r="P25" s="9"/>
     </row>
     <row r="26" spans="1:16" ht="13.2">
-      <c r="A26" s="15" t="s">
-        <v>38</v>
-      </c>
+      <c r="A26" s="15"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>97</v>
-      </c>
+      <c r="C26" s="17"/>
+      <c r="D26" s="18"/>
       <c r="E26" s="19"/>
       <c r="F26" s="20"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
-      <c r="O26" s="8"/>
+      <c r="K26" s="40"/>
+      <c r="L26" s="41"/>
+      <c r="M26" s="41"/>
+      <c r="N26" s="41"/>
+      <c r="O26" s="42"/>
       <c r="P26" s="9"/>
     </row>
     <row r="27" spans="1:16" ht="13.2">
-      <c r="A27" s="15" t="s">
-        <v>39</v>
-      </c>
+      <c r="A27" s="15"/>
       <c r="B27" s="16"/>
-      <c r="C27" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>98</v>
-      </c>
+      <c r="C27" s="17"/>
+      <c r="D27" s="18"/>
       <c r="E27" s="19"/>
       <c r="F27" s="20"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="8"/>
+      <c r="K27" s="40"/>
+      <c r="L27" s="41"/>
+      <c r="M27" s="41"/>
+      <c r="N27" s="41"/>
+      <c r="O27" s="42"/>
       <c r="P27" s="9"/>
     </row>
     <row r="28" spans="1:16" ht="13.2">
-      <c r="A28" s="15" t="s">
-        <v>40</v>
-      </c>
+      <c r="A28" s="15"/>
       <c r="B28" s="16"/>
-      <c r="C28" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="D28" s="18" t="s">
-        <v>99</v>
-      </c>
+      <c r="C28" s="17"/>
+      <c r="D28" s="18"/>
       <c r="E28" s="19"/>
       <c r="F28" s="20"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
       <c r="I28" s="7"/>
       <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
+      <c r="K28" s="40"/>
+      <c r="L28" s="41"/>
+      <c r="M28" s="41"/>
+      <c r="N28" s="41"/>
+      <c r="O28" s="42"/>
       <c r="P28" s="9"/>
     </row>
     <row r="29" spans="1:16" ht="13.2">
-      <c r="A29" s="15" t="s">
-        <v>41</v>
-      </c>
+      <c r="A29" s="15"/>
       <c r="B29" s="16"/>
-      <c r="C29" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="D29" s="18" t="s">
-        <v>100</v>
-      </c>
+      <c r="C29" s="17"/>
+      <c r="D29" s="18"/>
       <c r="E29" s="19"/>
       <c r="F29" s="20"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7"/>
-      <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
+      <c r="K29" s="40"/>
+      <c r="L29" s="41"/>
+      <c r="M29" s="41"/>
+      <c r="N29" s="41"/>
+      <c r="O29" s="42"/>
       <c r="P29" s="9"/>
     </row>
     <row r="30" spans="1:16" ht="13.2">
-      <c r="A30" s="15" t="s">
-        <v>42</v>
-      </c>
+      <c r="A30" s="15"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="D30" s="18" t="s">
-        <v>101</v>
-      </c>
+      <c r="C30" s="17"/>
+      <c r="D30" s="18"/>
       <c r="E30" s="19"/>
       <c r="F30" s="20"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="7"/>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
-      <c r="L30" s="7"/>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
+      <c r="K30" s="40"/>
+      <c r="L30" s="41"/>
+      <c r="M30" s="41"/>
+      <c r="N30" s="41"/>
+      <c r="O30" s="42"/>
       <c r="P30" s="9"/>
     </row>
     <row r="31" spans="1:16" ht="13.2">
-      <c r="A31" s="15" t="s">
-        <v>43</v>
-      </c>
+      <c r="A31" s="15"/>
       <c r="B31" s="16"/>
-      <c r="C31" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>102</v>
-      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="18"/>
       <c r="E31" s="19"/>
       <c r="F31" s="20"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="29"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="8"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="40"/>
+      <c r="L31" s="41"/>
+      <c r="M31" s="41"/>
+      <c r="N31" s="41"/>
+      <c r="O31" s="42"/>
       <c r="P31" s="9"/>
     </row>
     <row r="32" spans="1:16" ht="13.2">
@@ -2405,15 +1994,19 @@
       <c r="D32" s="18"/>
       <c r="E32" s="19"/>
       <c r="F32" s="20"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="29"/>
-      <c r="J32" s="29"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+      <c r="K32" s="40"/>
+      <c r="L32" s="41"/>
+      <c r="M32" s="41"/>
+      <c r="N32" s="41"/>
+      <c r="O32" s="42"/>
       <c r="P32" s="9"/>
     </row>
     <row r="33" spans="1:16" ht="13.2">
@@ -2423,36 +2016,44 @@
       <c r="D33" s="18"/>
       <c r="E33" s="19"/>
       <c r="F33" s="20"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="29"/>
-      <c r="J33" s="29"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+      <c r="O33" s="42"/>
       <c r="P33" s="9"/>
     </row>
-    <row r="34" spans="1:16" ht="13.2">
-      <c r="A34" s="32"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="29"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="30"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
+    <row r="34" spans="1:16" ht="13.8" thickBot="1">
+      <c r="A34" s="29"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="34"/>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34" s="7"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="40"/>
+      <c r="L34" s="41"/>
+      <c r="M34" s="41"/>
+      <c r="N34" s="41"/>
+      <c r="O34" s="42"/>
       <c r="P34" s="9"/>
     </row>
-    <row r="35" spans="1:16" ht="13.2">
+    <row r="35" spans="1:16" ht="13.8" thickTop="1">
       <c r="A35" s="7"/>
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
@@ -2461,13 +2062,13 @@
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
-      <c r="I35" s="29"/>
-      <c r="J35" s="29"/>
-      <c r="K35" s="38"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="40"/>
+      <c r="L35" s="41"/>
+      <c r="M35" s="41"/>
+      <c r="N35" s="41"/>
+      <c r="O35" s="42"/>
       <c r="P35" s="9"/>
     </row>
     <row r="36" spans="1:16" ht="13.2">
@@ -2481,11 +2082,11 @@
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="7"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
+      <c r="K36" s="40"/>
+      <c r="L36" s="41"/>
+      <c r="M36" s="41"/>
+      <c r="N36" s="41"/>
+      <c r="O36" s="42"/>
       <c r="P36" s="9"/>
     </row>
     <row r="37" spans="1:16" ht="13.2">
@@ -2499,11 +2100,11 @@
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
-      <c r="K37" s="8"/>
-      <c r="L37" s="8"/>
-      <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
+      <c r="K37" s="40"/>
+      <c r="L37" s="41"/>
+      <c r="M37" s="41"/>
+      <c r="N37" s="41"/>
+      <c r="O37" s="42"/>
       <c r="P37" s="9"/>
     </row>
     <row r="38" spans="1:16" ht="13.2">
@@ -2517,11 +2118,11 @@
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="7"/>
-      <c r="K38" s="8"/>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
+      <c r="K38" s="40"/>
+      <c r="L38" s="41"/>
+      <c r="M38" s="41"/>
+      <c r="N38" s="41"/>
+      <c r="O38" s="42"/>
       <c r="P38" s="9"/>
     </row>
     <row r="39" spans="1:16" ht="13.2">
@@ -2535,11 +2136,11 @@
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="7"/>
-      <c r="K39" s="8"/>
-      <c r="L39" s="8"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
+      <c r="K39" s="40"/>
+      <c r="L39" s="41"/>
+      <c r="M39" s="41"/>
+      <c r="N39" s="41"/>
+      <c r="O39" s="42"/>
       <c r="P39" s="9"/>
     </row>
     <row r="40" spans="1:16" ht="13.2">
@@ -2553,11 +2154,11 @@
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
       <c r="J40" s="7"/>
-      <c r="K40" s="8"/>
-      <c r="L40" s="8"/>
-      <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
+      <c r="K40" s="40"/>
+      <c r="L40" s="41"/>
+      <c r="M40" s="41"/>
+      <c r="N40" s="41"/>
+      <c r="O40" s="42"/>
       <c r="P40" s="9"/>
     </row>
     <row r="41" spans="1:16" ht="13.2">
@@ -2571,11 +2172,11 @@
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
       <c r="J41" s="7"/>
-      <c r="K41" s="8"/>
-      <c r="L41" s="8"/>
-      <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="8"/>
+      <c r="K41" s="40"/>
+      <c r="L41" s="41"/>
+      <c r="M41" s="41"/>
+      <c r="N41" s="41"/>
+      <c r="O41" s="42"/>
       <c r="P41" s="9"/>
     </row>
     <row r="42" spans="1:16" ht="13.2">
@@ -2589,11 +2190,11 @@
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
       <c r="J42" s="7"/>
-      <c r="K42" s="8"/>
-      <c r="L42" s="8"/>
-      <c r="M42" s="8"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="8"/>
+      <c r="K42" s="40"/>
+      <c r="L42" s="41"/>
+      <c r="M42" s="41"/>
+      <c r="N42" s="41"/>
+      <c r="O42" s="42"/>
       <c r="P42" s="9"/>
     </row>
     <row r="43" spans="1:16" ht="13.2">
@@ -2607,14 +2208,14 @@
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
       <c r="J43" s="7"/>
-      <c r="K43" s="8"/>
-      <c r="L43" s="8"/>
-      <c r="M43" s="8"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="8"/>
+      <c r="K43" s="40"/>
+      <c r="L43" s="41"/>
+      <c r="M43" s="41"/>
+      <c r="N43" s="41"/>
+      <c r="O43" s="42"/>
       <c r="P43" s="9"/>
     </row>
-    <row r="44" spans="1:16" ht="13.2">
+    <row r="44" spans="1:16" ht="13.8" thickBot="1">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -2625,14 +2226,14 @@
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
       <c r="J44" s="7"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="8"/>
-      <c r="M44" s="8"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
+      <c r="K44" s="43"/>
+      <c r="L44" s="44"/>
+      <c r="M44" s="44"/>
+      <c r="N44" s="44"/>
+      <c r="O44" s="45"/>
       <c r="P44" s="9"/>
     </row>
-    <row r="45" spans="1:16" ht="13.2">
+    <row r="45" spans="1:16" ht="13.8" thickTop="1">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
@@ -19860,20 +19461,27 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="L3:P3"/>
-    <mergeCell ref="L4:P23"/>
+    <mergeCell ref="K24:O24"/>
+    <mergeCell ref="K25:O44"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" prompt="Name must be a full name formatted as &quot;first last&quot;" sqref="G2 A2:A101 C2:C101 E2:E101" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations xWindow="824" yWindow="505" count="4">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" prompt="Name must be a full name formatted as &quot;first last&quot;" sqref="I2 A2:A101 C2:C101 E2:E101" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>NOT(ISERROR(SEARCH((" "),(A2))))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Kindergarten,1st grade,2nd grade,3rd grade,4th grade,5th grade"</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" prompt="Enter a valid email" sqref="D2:D1001 F2:F1001" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>IFERROR(ISEMAIL(D2), TRUE)</formula1>
     </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter a valid Tap Count (0 to Start)" sqref="G2:H34" xr:uid="{ED882FBB-04EE-42DC-971B-8064C4A8337B}">
+      <formula1>0</formula1>
+    </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{E514448C-6386-4D0B-BACE-B9D532082098}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>